<commit_message>
Update G4_L_QA02-Casos de Pruebas.xlsx
</commit_message>
<xml_diff>
--- a/IMPLANTACION/G4_L_QA02-Casos de Pruebas.xlsx
+++ b/IMPLANTACION/G4_L_QA02-Casos de Pruebas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kcalm\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6024496B-BB21-4489-80C2-E8CF484CBF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{55A52055-3DBA-48BB-8ADC-F1B79FFBAEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="98">
   <si>
     <t>Created By:</t>
   </si>
@@ -95,9 +95,6 @@
     <t xml:space="preserve">El usuario podra ingresar al sistema  </t>
   </si>
   <si>
-    <t xml:space="preserve">1. Colocar las credenciales dadas y darle al boton de inicio de sesion. </t>
-  </si>
-  <si>
     <t>Alta</t>
   </si>
   <si>
@@ -116,25 +113,7 @@
     <t xml:space="preserve"> Validar al ingresar sesion</t>
   </si>
   <si>
-    <t>1. Colocar todo tipo de valores para validar que al iniciar sesion dio error.</t>
-  </si>
-  <si>
-    <t>Al colocar cualquier tipo de valor para verificar que no lo deja ingresar le de un mensaje de error</t>
-  </si>
-  <si>
-    <t>Verificar la opcion de olvidar contrasena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muestre un mensaje con el usuario y la contrasena </t>
-  </si>
-  <si>
     <t>Usuarios</t>
-  </si>
-  <si>
-    <t>Ingresar datos de forma exitosa</t>
-  </si>
-  <si>
-    <t>Verificar el usuario colocando la cedula</t>
   </si>
   <si>
     <t>Seleccionar un usuario de la tabla y lo modifiques</t>
@@ -148,19 +127,6 @@
   </si>
   <si>
     <t>que se modifique los datos de forma exitora</t>
-  </si>
-  <si>
-    <t>Seleccionar un usuario de la tabla y lo elimines</t>
-  </si>
-  <si>
-    <t>seleccionar un usuario y que en los campos pueda ser eliminado</t>
-  </si>
-  <si>
-    <t>1. Seleccionar algun registro de la tabla .
-2. eliminar el registro en el boton eliminar</t>
-  </si>
-  <si>
-    <t>Desactivar un usuario de forma exitosa</t>
   </si>
   <si>
     <t>Buscar un usuario por el nombre o por cedula</t>
@@ -177,9 +143,6 @@
   </si>
   <si>
     <t>Roles</t>
-  </si>
-  <si>
-    <t>1. Agregar nuevos roles</t>
   </si>
   <si>
     <t>1. Si colocas datos, y te equivocaste en todo darle clic en el boton de nuevo.
@@ -208,35 +171,13 @@
 Pass =admin123                                                            </t>
   </si>
   <si>
-    <t>Mostrar el panel inical.</t>
-  </si>
-  <si>
-    <t>Usar un correo gmai para verificar que le devuelva la contrasena y el usuario para ingresar</t>
-  </si>
-  <si>
-    <t>1.Colocar el campo el email adecuado @gmail  
-2.Darle al boton de recuperar contrasena</t>
-  </si>
-  <si>
     <t xml:space="preserve">El sistema debe permitir registrar, editar y eliminar información de los usuarios </t>
   </si>
   <si>
     <t>El administrador registra un nuevo ingreso o edita informacion comprobada.</t>
   </si>
   <si>
-    <t>colocar la cedula y verifica los credenciales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Colocar la cedula </t>
-  </si>
-  <si>
     <t>Se requiere llenar los campos establecidos</t>
-  </si>
-  <si>
-    <t>1. Seleccionar agregar nuevo.</t>
-  </si>
-  <si>
-    <t>Se agregue de forma exitosa, lleando los campos requeridos con sus datos</t>
   </si>
   <si>
     <t>Categorias</t>
@@ -328,6 +269,74 @@
   <si>
     <t>Facultad de Farmacia</t>
   </si>
+  <si>
+    <t>1. Colocar las credenciales Presionar el boton "Iniciar Sesión".</t>
+  </si>
+  <si>
+    <t>Autenticación exitosa, redirección al panel principal</t>
+  </si>
+  <si>
+    <t>Digitar credenciales erróneas (ej. correo inexistente o clave incorrecta) y presionar "Iniciar Sesión".</t>
+  </si>
+  <si>
+    <t>Al colocar cualquier tipo de valor para verificar que no ingresa, muestra "Correo o contraseña incorrectos".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificar campos obligatorios para nuevo registro </t>
+  </si>
+  <si>
+    <t xml:space="preserve">no colocar credenciales y verificar el registro </t>
+  </si>
+  <si>
+    <t>Iniciaremos sesión como Administrador y entraremos al formulario de Crear Usuario</t>
+  </si>
+  <si>
+    <t>Ingresar datos sin éxito por campos vacios</t>
+  </si>
+  <si>
+    <t>iniciar sesion con el perfil de administrador</t>
+  </si>
+  <si>
+    <t>Automated</t>
+  </si>
+  <si>
+    <t>Buscar un rol por el nombre ocedula</t>
+  </si>
+  <si>
+    <t>Buscar un rol por el nombre o por cedula</t>
+  </si>
+  <si>
+    <t>1. Digitar un rol por el codigo o cedula.
+.</t>
+  </si>
+  <si>
+    <t>Existir una categoria previamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buscar una categoria por el nombre </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Digitar una categoria por el nombre.
+</t>
+  </si>
+  <si>
+    <t>Vista detallada de la categoria</t>
+  </si>
+  <si>
+    <t>Existir un registro de Categoria</t>
+  </si>
+  <si>
+    <t>seleccionar los detalles de alguna catgegoria en la tabla de registros</t>
+  </si>
+  <si>
+    <t>Vista de detalles para la categoria</t>
+  </si>
+  <si>
+    <t>Tener un registro previo de Docente</t>
+  </si>
+  <si>
+    <t>Tener un registro previo de Director</t>
+  </si>
 </sst>
 </file>
 
@@ -382,7 +391,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,6 +401,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -449,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -490,6 +505,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -794,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="D2" s="17"/>
       <c r="E2" s="1"/>
@@ -901,7 +919,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="D5" s="17"/>
       <c r="E5" s="1"/>
@@ -1036,33 +1054,33 @@
         <v>18</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="F8" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="I8" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J8" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="K8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K8" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L8" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M8" s="6"/>
       <c r="N8" s="8"/>
       <c r="O8" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
@@ -1090,36 +1108,36 @@
         <v>2</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="F9" s="7" t="s">
-        <v>26</v>
+        <v>78</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>27</v>
+        <v>79</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I9" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J9" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="K9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K9" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L9" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M9" s="5"/>
       <c r="N9" s="8"/>
       <c r="O9" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
@@ -1141,42 +1159,42 @@
     <row r="10" spans="1:31" ht="59.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
       <c r="B10" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="5">
-        <v>3</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>56</v>
+        <v>25</v>
+      </c>
+      <c r="C10" s="6">
+        <v>1</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>84</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>29</v>
+        <v>83</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I10" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J10" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="14" t="s">
+      <c r="K10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>22</v>
+      <c r="L10" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="8"/>
-      <c r="O10" s="5" t="s">
-        <v>22</v>
+      <c r="O10" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
@@ -1198,40 +1216,42 @@
     <row r="11" spans="1:31" ht="61.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
       <c r="B11" s="12" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C11" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="6"/>
+        <v>80</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>81</v>
+      </c>
       <c r="F11" s="7" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I11" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="K11" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K11" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L11" s="6" t="s">
-        <v>22</v>
+      <c r="L11" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="M11" s="5"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="6" t="s">
-        <v>22</v>
+      <c r="O11" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
@@ -1250,45 +1270,45 @@
       <c r="AD11" s="1"/>
       <c r="AE11" s="1"/>
     </row>
-    <row r="12" spans="1:31" ht="24" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:31" ht="48" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
       <c r="B12" s="12" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C12" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I12" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J12" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="K12" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K12" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L12" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="8"/>
       <c r="O12" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P12" s="1"/>
       <c r="Q12" s="1"/>
@@ -1310,42 +1330,42 @@
     <row r="13" spans="1:31" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="6">
+        <v>4</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="6">
-        <v>3</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="H13" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I13" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J13" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J13" s="14" t="s">
+      <c r="K13" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K13" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>22</v>
+      <c r="L13" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="M13" s="5"/>
       <c r="N13" s="8"/>
-      <c r="O13" s="5" t="s">
-        <v>22</v>
+      <c r="O13" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
@@ -1364,45 +1384,45 @@
       <c r="AD13" s="1"/>
       <c r="AE13" s="1"/>
     </row>
-    <row r="14" spans="1:31" ht="48" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
       <c r="B14" s="12" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C14" s="6">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>37</v>
+        <v>87</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>39</v>
+        <v>88</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I14" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J14" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J14" s="14" t="s">
+      <c r="K14" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K14" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L14" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M14" s="5"/>
       <c r="N14" s="8"/>
       <c r="O14" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P14" s="1"/>
       <c r="Q14" s="1"/>
@@ -1421,45 +1441,45 @@
       <c r="AD14" s="1"/>
       <c r="AE14" s="1"/>
     </row>
-    <row r="15" spans="1:31" ht="48" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="12" t="s">
-        <v>30</v>
+      <c r="B15" s="18" t="s">
+        <v>34</v>
       </c>
       <c r="C15" s="6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="I15" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J15" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J15" s="14" t="s">
+      <c r="K15" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K15" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>22</v>
+      <c r="L15" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="M15" s="5"/>
       <c r="N15" s="8"/>
-      <c r="O15" s="6" t="s">
-        <v>22</v>
+      <c r="O15" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="P15" s="1"/>
       <c r="Q15" s="1"/>
@@ -1478,45 +1498,45 @@
       <c r="AD15" s="1"/>
       <c r="AE15" s="1"/>
     </row>
-    <row r="16" spans="1:31" ht="36" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:31" ht="48" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
       <c r="B16" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C16" s="6">
         <v>1</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J16" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K16" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I16" s="5" t="s">
+      <c r="L16" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J16" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K16" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>22</v>
       </c>
       <c r="M16" s="5"/>
       <c r="N16" s="8"/>
-      <c r="O16" s="5" t="s">
-        <v>22</v>
+      <c r="O16" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="P16" s="1"/>
       <c r="Q16" s="1"/>
@@ -1538,7 +1558,7 @@
     <row r="17" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
       <c r="B17" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="6">
         <v>2</v>
@@ -1547,33 +1567,33 @@
         <v>49</v>
       </c>
       <c r="E17" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J17" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K17" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I17" s="5" t="s">
+      <c r="L17" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J17" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K17" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L17" s="5" t="s">
-        <v>22</v>
       </c>
       <c r="M17" s="5"/>
       <c r="N17" s="8"/>
-      <c r="O17" s="5" t="s">
-        <v>22</v>
+      <c r="O17" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
@@ -1595,42 +1615,42 @@
     <row r="18" spans="1:31" ht="48.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
       <c r="B18" s="12" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="C18" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J18" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K18" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I18" s="5" t="s">
+      <c r="L18" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J18" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K18" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M18" s="5"/>
       <c r="N18" s="8"/>
       <c r="O18" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
@@ -1652,43 +1672,37 @@
     <row r="19" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
       <c r="B19" s="12" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="C19" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="E19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J19" s="14"/>
+      <c r="K19" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K19" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L19" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="L19" s="6"/>
       <c r="M19" s="5"/>
       <c r="N19" s="8"/>
-      <c r="O19" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="O19" s="6"/>
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
@@ -1709,43 +1723,37 @@
     <row r="20" spans="1:31" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
       <c r="B20" s="12" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="C20" s="6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J20" s="14"/>
+      <c r="K20" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F20" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I20" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="J20" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K20" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L20" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="L20" s="6"/>
       <c r="M20" s="5"/>
       <c r="N20" s="8"/>
-      <c r="O20" s="6" t="s">
-        <v>22</v>
-      </c>
+      <c r="O20" s="6"/>
       <c r="P20" s="1"/>
       <c r="Q20" s="1"/>
       <c r="R20" s="1"/>
@@ -1766,42 +1774,42 @@
     <row r="21" spans="1:31" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
       <c r="B21" s="12" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C21" s="6">
         <v>1</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J21" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K21" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F21" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I21" s="5" t="s">
+      <c r="L21" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K21" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L21" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M21" s="5"/>
       <c r="N21" s="8"/>
       <c r="O21" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
@@ -1823,42 +1831,42 @@
     <row r="22" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
       <c r="B22" s="12" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C22" s="6">
         <v>2</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J22" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K22" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F22" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I22" s="5" t="s">
+      <c r="L22" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J22" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K22" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L22" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M22" s="5"/>
       <c r="N22" s="8"/>
       <c r="O22" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
@@ -1880,42 +1888,42 @@
     <row r="23" spans="1:31" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
       <c r="B23" s="12" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C23" s="6">
         <v>3</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>72</v>
+        <v>53</v>
       </c>
       <c r="E23" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I23" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J23" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K23" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F23" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G23" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H23" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I23" s="5" t="s">
+      <c r="L23" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J23" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K23" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L23" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M23" s="5"/>
       <c r="N23" s="8"/>
       <c r="O23" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
@@ -1937,42 +1945,42 @@
     <row r="24" spans="1:31" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
       <c r="B24" s="12" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C24" s="6">
         <v>4</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J24" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K24" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G24" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I24" s="5" t="s">
+      <c r="L24" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K24" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M24" s="5"/>
       <c r="N24" s="8"/>
       <c r="O24" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
@@ -1994,42 +2002,42 @@
     <row r="25" spans="1:31" ht="24" x14ac:dyDescent="0.2">
       <c r="A25" s="1"/>
       <c r="B25" s="12" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="C25" s="6">
         <v>5</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I25" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J25" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K25" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F25" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G25" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H25" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I25" s="5" t="s">
+      <c r="L25" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J25" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K25" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M25" s="5"/>
       <c r="N25" s="8"/>
       <c r="O25" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
@@ -2051,42 +2059,42 @@
     <row r="26" spans="1:31" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="12" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C26" s="6">
         <v>1</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E26" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J26" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K26" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I26" s="5" t="s">
+      <c r="L26" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J26" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K26" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L26" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M26" s="5"/>
       <c r="N26" s="8"/>
       <c r="O26" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
@@ -2108,42 +2116,40 @@
     <row r="27" spans="1:31" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
       <c r="B27" s="12" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C27" s="6">
         <v>2</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E27" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E27" s="6"/>
+      <c r="F27" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J27" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K27" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H27" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I27" s="5" t="s">
+      <c r="L27" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K27" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L27" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M27" s="5"/>
       <c r="N27" s="8"/>
       <c r="O27" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
@@ -2165,42 +2171,42 @@
     <row r="28" spans="1:31" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1"/>
       <c r="B28" s="12" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C28" s="6">
         <v>3</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E28" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J28" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K28" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I28" s="5" t="s">
+      <c r="L28" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J28" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K28" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L28" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M28" s="5"/>
       <c r="N28" s="8"/>
       <c r="O28" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
@@ -2222,42 +2228,42 @@
     <row r="29" spans="1:31" ht="39" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1"/>
       <c r="B29" s="12" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C29" s="6">
         <v>4</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J29" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K29" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G29" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H29" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I29" s="5" t="s">
+      <c r="L29" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J29" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K29" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L29" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M29" s="5"/>
       <c r="N29" s="8"/>
       <c r="O29" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
@@ -2279,42 +2285,42 @@
     <row r="30" spans="1:31" ht="24" x14ac:dyDescent="0.2">
       <c r="A30" s="1"/>
       <c r="B30" s="12" t="s">
-        <v>73</v>
+        <v>54</v>
       </c>
       <c r="C30" s="6">
         <v>5</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="E30" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="J30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K30" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F30" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I30" s="5" t="s">
+      <c r="L30" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J30" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K30" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L30" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M30" s="5"/>
       <c r="N30" s="8"/>
       <c r="O30" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
@@ -2336,42 +2342,40 @@
     <row r="31" spans="1:31" ht="48" x14ac:dyDescent="0.2">
       <c r="A31" s="1"/>
       <c r="B31" s="12" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C31" s="6">
         <v>1</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="6"/>
+      <c r="F31" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I31" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K31" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G31" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I31" s="5" t="s">
+      <c r="L31" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J31" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K31" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L31" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M31" s="5"/>
       <c r="N31" s="8"/>
       <c r="O31" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
@@ -2393,42 +2397,42 @@
     <row r="32" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A32" s="1"/>
       <c r="B32" s="12" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C32" s="6">
         <v>2</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="E32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H32" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K32" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F32" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I32" s="5" t="s">
+      <c r="L32" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J32" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K32" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M32" s="5"/>
       <c r="N32" s="8"/>
       <c r="O32" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
@@ -2450,42 +2454,42 @@
     <row r="33" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="B33" s="12" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C33" s="6">
         <v>3</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E33" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G33" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H33" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J33" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K33" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F33" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="H33" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I33" s="5" t="s">
+      <c r="L33" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J33" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K33" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L33" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M33" s="5"/>
       <c r="N33" s="8"/>
       <c r="O33" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
@@ -2507,42 +2511,42 @@
     <row r="34" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A34" s="1"/>
       <c r="B34" s="12" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C34" s="6">
         <v>4</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E34" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H34" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J34" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K34" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F34" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="G34" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I34" s="5" t="s">
+      <c r="L34" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J34" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K34" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L34" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M34" s="5"/>
       <c r="N34" s="8"/>
       <c r="O34" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
@@ -2564,42 +2568,42 @@
     <row r="35" spans="1:31" ht="24" x14ac:dyDescent="0.2">
       <c r="A35" s="1"/>
       <c r="B35" s="12" t="s">
-        <v>75</v>
+        <v>56</v>
       </c>
       <c r="C35" s="6">
         <v>5</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="E35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J35" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="K35" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F35" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I35" s="5" t="s">
+      <c r="L35" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="J35" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K35" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="L35" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="M35" s="5"/>
       <c r="N35" s="8"/>
       <c r="O35" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
@@ -2621,42 +2625,42 @@
     <row r="36" spans="1:31" ht="60" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
       <c r="B36" s="15" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="C36" s="6">
         <v>1</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I36" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J36" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J36" s="14" t="s">
+      <c r="K36" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K36" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L36" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M36" s="5"/>
       <c r="N36" s="8"/>
       <c r="O36" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
@@ -2678,42 +2682,42 @@
     <row r="37" spans="1:31" ht="36" x14ac:dyDescent="0.2">
       <c r="A37" s="1"/>
       <c r="B37" s="15" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="C37" s="6">
         <v>2</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="H37" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I37" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I37" s="5" t="s">
+      <c r="J37" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="J37" s="14" t="s">
+      <c r="K37" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K37" s="13" t="s">
-        <v>23</v>
-      </c>
       <c r="L37" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M37" s="5"/>
       <c r="N37" s="8"/>
       <c r="O37" s="6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
@@ -34083,7 +34087,6 @@
       <c r="AE987" s="1"/>
     </row>
     <row r="988" spans="1:31" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A988" s="1"/>
       <c r="B988" s="1"/>
       <c r="C988" s="1"/>
       <c r="D988" s="1"/>

</xml_diff>